<commit_message>
Realización de script de comunicación entre la base de datos y el excel correcto, y corrección en la solicitud de reserva
</commit_message>
<xml_diff>
--- a/app_horarios/datos/excel/import.xlsx
+++ b/app_horarios/datos/excel/import.xlsx
@@ -5,35 +5,34 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usuario\Desktop\Ingeniería informática\4º Trabajo de Fin de Grado\Material TFG\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usuario\Desktop\Ingeniería informática\4º Trabajo de Fin de Grado\Trabajo-Fin-de-Grado-2025-2026\app_horarios\datos\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{3017ED77-2F17-4B0C-9184-641C590491F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB89CAAE-98C3-4103-A24C-C6D305CCA5BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="13" xr2:uid="{A94C5715-B1A2-4C5E-A79C-F50E817DAD22}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="8" activeTab="16" xr2:uid="{A94C5715-B1A2-4C5E-A79C-F50E817DAD22}"/>
   </bookViews>
   <sheets>
-    <sheet name="AULA" sheetId="1" r:id="rId1"/>
-    <sheet name="RESPONSABLE" sheetId="2" r:id="rId2"/>
-    <sheet name="RESERVA" sheetId="3" r:id="rId3"/>
-    <sheet name="RESERVA_PUNTUAL" sheetId="4" r:id="rId4"/>
-    <sheet name="RESERVA_PERIODICA" sheetId="5" r:id="rId5"/>
-    <sheet name="DOCENTE" sheetId="6" r:id="rId6"/>
-    <sheet name="ASIGNATURAS" sheetId="7" r:id="rId7"/>
-    <sheet name="IMPARTE" sheetId="8" r:id="rId8"/>
-    <sheet name="GRADO" sheetId="9" r:id="rId9"/>
-    <sheet name="GRUPO" sheetId="10" r:id="rId10"/>
-    <sheet name="CURSO" sheetId="11" r:id="rId11"/>
-    <sheet name="SEMESTRE" sheetId="12" r:id="rId12"/>
-    <sheet name="DIA" sheetId="13" r:id="rId13"/>
-    <sheet name="LECTIVO" sheetId="14" r:id="rId14"/>
-    <sheet name="CAMBIO_DOCENCIA" sheetId="18" r:id="rId15"/>
-    <sheet name="EXAMEN" sheetId="15" r:id="rId16"/>
-    <sheet name="FESTIVO" sheetId="16" r:id="rId17"/>
-    <sheet name="TFG" sheetId="17" r:id="rId18"/>
+    <sheet name="aula" sheetId="1" r:id="rId1"/>
+    <sheet name="responsable" sheetId="2" r:id="rId2"/>
+    <sheet name="reserva" sheetId="3" r:id="rId3"/>
+    <sheet name="reserva_puntual" sheetId="4" r:id="rId4"/>
+    <sheet name="reserva_periodica" sheetId="5" r:id="rId5"/>
+    <sheet name="docente" sheetId="6" r:id="rId6"/>
+    <sheet name="asignaturas" sheetId="7" r:id="rId7"/>
+    <sheet name="imparte" sheetId="8" r:id="rId8"/>
+    <sheet name="grado" sheetId="9" r:id="rId9"/>
+    <sheet name="grupo" sheetId="10" r:id="rId10"/>
+    <sheet name="curso" sheetId="11" r:id="rId11"/>
+    <sheet name="semestre" sheetId="12" r:id="rId12"/>
+    <sheet name="dia" sheetId="13" r:id="rId13"/>
+    <sheet name="lectivo" sheetId="14" r:id="rId14"/>
+    <sheet name="cambio_docencia" sheetId="18" r:id="rId15"/>
+    <sheet name="examen" sheetId="15" r:id="rId16"/>
+    <sheet name="festivo" sheetId="16" r:id="rId17"/>
+    <sheet name="tfg" sheetId="17" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -463,12 +462,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -886,7 +884,7 @@
         <v>60</v>
       </c>
       <c r="L2">
-        <f>GRADO!$A$2</f>
+        <f>grado!$A$2</f>
         <v>281</v>
       </c>
       <c r="M2">
@@ -925,7 +923,7 @@
         <v>40</v>
       </c>
       <c r="L3">
-        <f>GRADO!$A$2</f>
+        <f>grado!$A$2</f>
         <v>281</v>
       </c>
       <c r="M3">
@@ -967,7 +965,7 @@
         <v>64</v>
       </c>
       <c r="L4">
-        <f>GRADO!A3</f>
+        <f>grado!A3</f>
         <v>147</v>
       </c>
       <c r="M4">
@@ -1006,7 +1004,7 @@
         <v>20</v>
       </c>
       <c r="L5">
-        <f>GRADO!A5</f>
+        <f>grado!A5</f>
         <v>291</v>
       </c>
       <c r="M5">
@@ -5286,7 +5284,7 @@
       <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -5347,7 +5345,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
-        <v>45005</v>
+        <v>46101</v>
       </c>
       <c r="B7" t="s">
         <v>110</v>
@@ -5876,7 +5874,7 @@
         <v>6</v>
       </c>
       <c r="G2">
-        <f>GRADO!$A$2</f>
+        <f>grado!$A$2</f>
         <v>281</v>
       </c>
       <c r="H2" t="s">
@@ -5906,7 +5904,7 @@
         <v>6</v>
       </c>
       <c r="G3">
-        <f>GRADO!$A$2</f>
+        <f>grado!$A$2</f>
         <v>281</v>
       </c>
       <c r="H3" t="s">
@@ -5936,7 +5934,7 @@
         <v>6</v>
       </c>
       <c r="G4">
-        <f>GRADO!$A$2</f>
+        <f>grado!$A$2</f>
         <v>281</v>
       </c>
       <c r="H4" t="s">

</xml_diff>

<commit_message>
Correción color de botones, y que aparezca en las solicitudes pendientes los datos que no salían de las reservas
</commit_message>
<xml_diff>
--- a/app_horarios/datos/excel/import.xlsx
+++ b/app_horarios/datos/excel/import.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usuario\Desktop\Ingeniería informática\4º Trabajo de Fin de Grado\Trabajo-Fin-de-Grado-2025-2026\app_horarios\datos\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB89CAAE-98C3-4103-A24C-C6D305CCA5BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F04CE34-DCFE-4F81-BEC8-5616F07E035C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="8" activeTab="16" xr2:uid="{A94C5715-B1A2-4C5E-A79C-F50E817DAD22}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{A94C5715-B1A2-4C5E-A79C-F50E817DAD22}"/>
   </bookViews>
   <sheets>
     <sheet name="aula" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="122">
   <si>
     <t>NOMBRE</t>
   </si>
@@ -404,6 +404,21 @@
   </si>
   <si>
     <t>San Pedro y San Pablo</t>
+  </si>
+  <si>
+    <t>NUM_ORDENADORES_SOLICITADOS</t>
+  </si>
+  <si>
+    <t>ALTAVOCES_SOLICITADOS</t>
+  </si>
+  <si>
+    <t>PROYECTOR_SOLICITADO</t>
+  </si>
+  <si>
+    <t>CAMARA_SOLICITADA</t>
+  </si>
+  <si>
+    <t>ENCHUFES_SOLICITADOS</t>
   </si>
 </sst>
 </file>
@@ -5652,16 +5667,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E078E57-8342-4B12-A2BC-28272F94D4A6}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -5672,21 +5685,15 @@
         <v>19</v>
       </c>
       <c r="D1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I1" t="s">
         <v>25</v>
       </c>
     </row>
@@ -5697,13 +5704,20 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CCFE1E2-1F6B-4D5B-934A-380C58E17123}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -5711,13 +5725,34 @@
         <v>28</v>
       </c>
       <c r="C1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" t="s">
         <v>29</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>30</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>31</v>
+      </c>
+      <c r="G1" t="s">
+        <v>117</v>
+      </c>
+      <c r="H1" t="s">
+        <v>118</v>
+      </c>
+      <c r="I1" t="s">
+        <v>119</v>
+      </c>
+      <c r="J1" t="s">
+        <v>120</v>
+      </c>
+      <c r="K1" t="s">
+        <v>121</v>
+      </c>
+      <c r="L1" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>